<commit_message>
Refactor genetic algorithm and evaluator for improved reporting and parameter handling; add Optuna integration for hyperparameter tuning
</commit_message>
<xml_diff>
--- a/Inputs_Doceleia_small.xlsx
+++ b/Inputs_Doceleia_small.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kaizen\Documents\tese\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE5AEEEA-485C-4649-9D9C-70B6CAD5BF9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DD3C7F4-9F38-4D26-9DCD-73C5A47648A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_ESTRUTURA" sheetId="2" r:id="rId1"/>
@@ -757,8 +757,30 @@
 </comments>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2143" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2145" uniqueCount="536">
   <si>
     <t>ESTRUTURA FÍSICA DO SISTEMA PRODUTIVO</t>
   </si>
@@ -2360,6 +2382,12 @@
   </si>
   <si>
     <t>unid_caixa</t>
+  </si>
+  <si>
+    <t>Familia</t>
+  </si>
+  <si>
+    <t>Monday</t>
   </si>
 </sst>
 </file>
@@ -2507,7 +2535,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2560,6 +2588,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2682,7 +2716,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2892,11 +2926,19 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="21">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -3629,26 +3671,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A2E0425D-8D3D-4317-A507-ADC777C31517}" name="Table4" displayName="Table4" ref="A4:Q192" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" tableBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A2E0425D-8D3D-4317-A507-ADC777C31517}" name="Table4" displayName="Table4" ref="A4:Q192" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18">
   <autoFilter ref="A4:Q192" xr:uid="{A2E0425D-8D3D-4317-A507-ADC777C31517}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{26D481BD-1A66-4F75-A5DB-835BDEAD35EC}" name="ref_id" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{AF3D888D-29CC-4818-9F37-35E1C095FEBC}" name="nome" dataDxfId="15"/>
-    <tableColumn id="21" xr3:uid="{A36D18E5-0E2F-48D2-A9EA-1667409CF7FA}" name="Unid_caixa" dataDxfId="14"/>
-    <tableColumn id="19" xr3:uid="{901BF69A-B9CB-436F-8A73-E52E627A4C44}" name="nao_produzir_segunda" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{73E06642-D2DC-4B3F-B7AE-6A99CF0B73CD}" name="família" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{47F7E5B0-45A6-4E01-8304-DD4D19A9E24E}" name="ativa" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{E576D14B-BDA0-4CA6-B2F4-097D5C1CE99B}" name="pode_L1" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{B29DBEC4-DD50-4914-98AC-30F025559FDC}" name="tempo_L1_prod_min (cadência de L1)" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{14DD02B2-C00E-494B-A8F3-3FFAE31BC4FB}" name="operadores_nec_L1_acab" dataDxfId="8"/>
-    <tableColumn id="13" xr3:uid="{89492EE9-DE84-43EE-B12E-2605FE3EAD79}" name="operadores_nec_L1_prod" dataDxfId="7"/>
-    <tableColumn id="14" xr3:uid="{780BF028-7B4E-42E1-B807-EDB2FB22CEE7}" name="pode_L2" dataDxfId="6"/>
-    <tableColumn id="15" xr3:uid="{FD12F15B-F3BE-48A4-B186-794E71F468D8}" name="tempo_L2_prod_min (cadência de L2)" dataDxfId="5"/>
-    <tableColumn id="16" xr3:uid="{2B695F9C-3774-41DD-8FE4-AF094E98B022}" name="tempo_L2_acab_min (cadência de L2)" dataDxfId="4"/>
-    <tableColumn id="20" xr3:uid="{46C45284-5F2B-442A-A3EB-D66468126784}" name="operadores_nec_L2_acab" dataDxfId="3"/>
-    <tableColumn id="17" xr3:uid="{1453032D-3307-46D2-BB7E-3D55B4D2E43D}" name="operadores_nec_L2_prod" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{5009F860-773A-42AE-9780-72CCCE321658}" name="kg" dataDxfId="1"/>
-    <tableColumn id="18" xr3:uid="{3939DDEA-30DE-43D1-B600-33ECEC5CD680}" name="euros" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{26D481BD-1A66-4F75-A5DB-835BDEAD35EC}" name="ref_id" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{AF3D888D-29CC-4818-9F37-35E1C095FEBC}" name="nome" dataDxfId="16"/>
+    <tableColumn id="21" xr3:uid="{A36D18E5-0E2F-48D2-A9EA-1667409CF7FA}" name="Unid_caixa" dataDxfId="15"/>
+    <tableColumn id="19" xr3:uid="{901BF69A-B9CB-436F-8A73-E52E627A4C44}" name="nao_produzir_segunda" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{73E06642-D2DC-4B3F-B7AE-6A99CF0B73CD}" name="família" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{47F7E5B0-45A6-4E01-8304-DD4D19A9E24E}" name="ativa" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{E576D14B-BDA0-4CA6-B2F4-097D5C1CE99B}" name="pode_L1" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{B29DBEC4-DD50-4914-98AC-30F025559FDC}" name="tempo_L1_prod_min (cadência de L1)" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{14DD02B2-C00E-494B-A8F3-3FFAE31BC4FB}" name="operadores_nec_L1_acab" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{89492EE9-DE84-43EE-B12E-2605FE3EAD79}" name="operadores_nec_L1_prod" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{780BF028-7B4E-42E1-B807-EDB2FB22CEE7}" name="pode_L2" dataDxfId="7"/>
+    <tableColumn id="15" xr3:uid="{FD12F15B-F3BE-48A4-B186-794E71F468D8}" name="tempo_L2_prod_min (cadência de L2)" dataDxfId="6"/>
+    <tableColumn id="16" xr3:uid="{2B695F9C-3774-41DD-8FE4-AF094E98B022}" name="tempo_L2_acab_min (cadência de L2)" dataDxfId="5"/>
+    <tableColumn id="20" xr3:uid="{46C45284-5F2B-442A-A3EB-D66468126784}" name="operadores_nec_L2_acab" dataDxfId="4"/>
+    <tableColumn id="17" xr3:uid="{1453032D-3307-46D2-BB7E-3D55B4D2E43D}" name="operadores_nec_L2_prod" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{5009F860-773A-42AE-9780-72CCCE321658}" name="kg" dataDxfId="2"/>
+    <tableColumn id="18" xr3:uid="{3939DDEA-30DE-43D1-B600-33ECEC5CD680}" name="euros" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4009,7 +4051,7 @@
         <v>474</v>
       </c>
       <c r="B4" s="31">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="C4" s="3"/>
     </row>
@@ -4018,7 +4060,7 @@
         <v>469</v>
       </c>
       <c r="B5" s="31">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="C5" s="3"/>
     </row>
@@ -18750,17 +18792,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="B1:L111"/>
+  <dimension ref="B1:N111"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14" style="6" customWidth="1"/>
     <col min="3" max="4" width="18" style="14" customWidth="1"/>
-    <col min="5" max="7" width="24.26953125" style="38" customWidth="1"/>
-    <col min="9" max="9" width="62.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="8" width="24.26953125" style="38" customWidth="1"/>
+    <col min="10" max="10" width="62.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:14" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B1" s="63" t="s">
         <v>36</v>
       </c>
@@ -18769,11 +18811,13 @@
       <c r="E1" s="62"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
-      <c r="H1">
-        <v>22.5</v>
-      </c>
-    </row>
-    <row r="2" spans="2:12" ht="35" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="H1" s="6"/>
+      <c r="I1">
+        <f>5*450/60</f>
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="2" spans="2:14" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="61" t="s">
         <v>404</v>
       </c>
@@ -18783,19 +18827,24 @@
       <c r="F2" s="59" t="s">
         <v>529</v>
       </c>
-      <c r="G2" s="58" t="e">
-        <f>SUM(F5,F8,#REF!,F9,F10,F12,F14,F15,F16,F20)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="G2" s="59"/>
+      <c r="H2" s="58">
+        <f>SUM(F5,F8,F9,F10,F12,F14,F15,F16,F18)</f>
+        <v>36.09394871794872</v>
+      </c>
+      <c r="I2" t="s">
         <v>531</v>
       </c>
-      <c r="I2" s="40" t="e">
-        <f>SUM(F6,F7,F11,#REF!,F13,F17)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="4" spans="2:12" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J2" s="40">
+        <f>SUM(F6,F7,F11,F13,F17,F19)</f>
+        <v>39.036189792663478</v>
+      </c>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="M3" s="75"/>
+      <c r="N3" s="75"/>
+    </row>
+    <row r="4" spans="2:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B4" s="35" t="s">
         <v>28</v>
       </c>
@@ -18811,9 +18860,16 @@
       <c r="F4" s="56" t="s">
         <v>530</v>
       </c>
-      <c r="G4" s="56"/>
-    </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="G4" s="56" t="s">
+        <v>534</v>
+      </c>
+      <c r="H4" s="56" t="s">
+        <v>535</v>
+      </c>
+      <c r="M4" s="75"/>
+      <c r="N4" s="75"/>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B5" s="34" t="s">
         <v>224</v>
       </c>
@@ -18821,7 +18877,7 @@
         <v>168</v>
       </c>
       <c r="D5" s="37">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="E5" s="60">
         <v>2</v>
@@ -18830,21 +18886,29 @@
         <f>(168*2)/(_xlfn.XLOOKUP(B5,Table4[ref_id],Table4[tempo_L1_prod_min (cadência de L1)]))</f>
         <v>1.8666666666666667</v>
       </c>
-      <c r="G5" s="34"/>
-      <c r="I5" s="55" t="s">
+      <c r="G5" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B5,Table4[ref_id],Table4[família])</f>
+        <v>NK</v>
+      </c>
+      <c r="H5" s="34" cm="1">
+        <f t="array" ref="H5">_xlfn.XLOOKUP(B5,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>1</v>
+      </c>
+      <c r="J5" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="J5" s="55" t="s">
+      <c r="K5" s="55" t="s">
         <v>224</v>
       </c>
-      <c r="K5" s="55" t="s">
+      <c r="L5" s="55" t="s">
         <v>406</v>
       </c>
-      <c r="L5" s="55" t="s">
+      <c r="M5" s="55" t="s">
         <v>527</v>
       </c>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N5" s="75"/>
+    </row>
+    <row r="6" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B6" s="34" t="s">
         <v>232</v>
       </c>
@@ -18852,30 +18916,38 @@
         <v>280</v>
       </c>
       <c r="D6" s="37">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="E6" s="60">
         <v>45</v>
       </c>
       <c r="F6" s="34">
-        <f>(100*E6/800)</f>
-        <v>5.625</v>
-      </c>
-      <c r="G6" s="34"/>
-      <c r="I6" s="55" t="s">
+        <f>(280*E6/800)</f>
+        <v>15.75</v>
+      </c>
+      <c r="G6" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B6,Table4[ref_id],Table4[família])</f>
+        <v>TM</v>
+      </c>
+      <c r="H6" s="34" cm="1">
+        <f t="array" ref="H6">_xlfn.XLOOKUP(B6,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>1</v>
+      </c>
+      <c r="J6" s="55" t="s">
         <v>56</v>
       </c>
-      <c r="J6" s="55" t="s">
+      <c r="K6" s="55" t="s">
         <v>232</v>
       </c>
-      <c r="K6" s="55" t="s">
-        <v>526</v>
-      </c>
       <c r="L6" s="55" t="s">
+        <v>406</v>
+      </c>
+      <c r="M6" s="55" t="s">
         <v>528</v>
       </c>
-    </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N6" s="75"/>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B7" s="34" t="s">
         <v>243</v>
       </c>
@@ -18883,30 +18955,38 @@
         <v>200</v>
       </c>
       <c r="D7" s="37">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="E7" s="60">
         <v>90</v>
       </c>
       <c r="F7" s="34">
-        <f>(50*E7/3456)</f>
-        <v>1.3020833333333333</v>
-      </c>
-      <c r="G7" s="34"/>
-      <c r="I7" s="55" t="s">
+        <f>(200*E7/3456)</f>
+        <v>5.208333333333333</v>
+      </c>
+      <c r="G7" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B7,Table4[ref_id],Table4[família])</f>
+        <v>MF</v>
+      </c>
+      <c r="H7" s="34" cm="1">
+        <f t="array" ref="H7">_xlfn.XLOOKUP(B7,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>0</v>
+      </c>
+      <c r="J7" s="55" t="s">
         <v>66</v>
       </c>
-      <c r="J7" s="55" t="s">
+      <c r="K7" s="55" t="s">
         <v>243</v>
       </c>
-      <c r="K7" s="55" t="s">
+      <c r="L7" s="55" t="s">
         <v>526</v>
       </c>
-      <c r="L7" s="55" t="s">
+      <c r="M7" s="55" t="s">
         <v>528</v>
       </c>
-    </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N7" s="75"/>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B8" s="34" t="s">
         <v>260</v>
       </c>
@@ -18914,7 +18994,7 @@
         <v>1000</v>
       </c>
       <c r="D8" s="37">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="E8" s="60">
         <v>4</v>
@@ -18923,21 +19003,29 @@
         <f>C8*E8/(_xlfn.XLOOKUP(B8,Table4[ref_id],Table4[tempo_L1_prod_min (cadência de L1)]))</f>
         <v>15.384615384615385</v>
       </c>
-      <c r="G8" s="34"/>
-      <c r="I8" s="55" t="s">
+      <c r="G8" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B8,Table4[ref_id],Table4[família])</f>
+        <v>TN</v>
+      </c>
+      <c r="H8" s="34" cm="1">
+        <f t="array" ref="H8">_xlfn.XLOOKUP(B8,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>1</v>
+      </c>
+      <c r="J8" s="55" t="s">
         <v>83</v>
       </c>
-      <c r="J8" s="55" t="s">
+      <c r="K8" s="55" t="s">
         <v>260</v>
       </c>
-      <c r="K8" s="55" t="s">
+      <c r="L8" s="55" t="s">
         <v>406</v>
       </c>
-      <c r="L8" s="55" t="s">
+      <c r="M8" s="55" t="s">
         <v>527</v>
       </c>
-    </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N8" s="75"/>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B9" s="34" t="s">
         <v>287</v>
       </c>
@@ -18945,7 +19033,7 @@
         <v>96</v>
       </c>
       <c r="D9" s="37">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="E9" s="60">
         <v>4</v>
@@ -18954,21 +19042,29 @@
         <f>C9*E9/(_xlfn.XLOOKUP(B9,Table4[ref_id],Table4[tempo_L1_prod_min (cadência de L1)]))</f>
         <v>1.92</v>
       </c>
-      <c r="G9" s="34"/>
-      <c r="I9" s="55" t="s">
+      <c r="G9" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B9,Table4[ref_id],Table4[família])</f>
+        <v>TR</v>
+      </c>
+      <c r="H9" s="34" cm="1">
+        <f t="array" ref="H9">_xlfn.XLOOKUP(B9,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>1</v>
+      </c>
+      <c r="J9" s="55" t="s">
         <v>84</v>
       </c>
-      <c r="J9" s="55" t="s">
+      <c r="K9" s="55" t="s">
         <v>261</v>
       </c>
-      <c r="K9" s="55" t="s">
+      <c r="L9" s="55" t="s">
         <v>510</v>
       </c>
-      <c r="L9" s="55" t="s">
+      <c r="M9" s="55" t="s">
         <v>527</v>
       </c>
-    </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N9" s="75"/>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B10" s="34" t="s">
         <v>298</v>
       </c>
@@ -18976,7 +19072,7 @@
         <v>96</v>
       </c>
       <c r="D10" s="37">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="E10" s="60">
         <v>4</v>
@@ -18985,21 +19081,29 @@
         <f>C10*E10/(_xlfn.XLOOKUP(B10,Table4[ref_id],Table4[tempo_L1_prod_min (cadência de L1)]))</f>
         <v>1.92</v>
       </c>
-      <c r="G10" s="34"/>
-      <c r="I10" s="55" t="s">
+      <c r="G10" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B10,Table4[ref_id],Table4[família])</f>
+        <v>TR</v>
+      </c>
+      <c r="H10" s="34" cm="1">
+        <f t="array" ref="H10">_xlfn.XLOOKUP(B10,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>1</v>
+      </c>
+      <c r="J10" s="55" t="s">
         <v>110</v>
       </c>
-      <c r="J10" s="55" t="s">
+      <c r="K10" s="55" t="s">
         <v>287</v>
       </c>
-      <c r="K10" s="55" t="s">
+      <c r="L10" s="55" t="s">
         <v>406</v>
       </c>
-      <c r="L10" s="55" t="s">
+      <c r="M10" s="55" t="s">
         <v>527</v>
       </c>
-    </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N10" s="75"/>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B11" s="34" t="s">
         <v>305</v>
       </c>
@@ -19016,21 +19120,29 @@
         <f>C11*E11/125</f>
         <v>4.6079999999999997</v>
       </c>
-      <c r="G11" s="34"/>
-      <c r="I11" s="55" t="s">
+      <c r="G11" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B11,Table4[ref_id],Table4[família])</f>
+        <v>DC</v>
+      </c>
+      <c r="H11" s="34" cm="1">
+        <f t="array" ref="H11">_xlfn.XLOOKUP(B11,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>1</v>
+      </c>
+      <c r="J11" s="55" t="s">
         <v>122</v>
       </c>
-      <c r="J11" s="55" t="s">
+      <c r="K11" s="55" t="s">
         <v>298</v>
       </c>
-      <c r="K11" s="55" t="s">
+      <c r="L11" s="55" t="s">
         <v>406</v>
       </c>
-      <c r="L11" s="55" t="s">
+      <c r="M11" s="55" t="s">
         <v>527</v>
       </c>
-    </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N11" s="75"/>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B12" s="34" t="s">
         <v>328</v>
       </c>
@@ -19038,7 +19150,7 @@
         <v>96</v>
       </c>
       <c r="D12" s="37">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="E12" s="60">
         <v>4</v>
@@ -19047,21 +19159,29 @@
         <f>C12*E12/(_xlfn.XLOOKUP(B12,Table4[ref_id],Table4[tempo_L1_prod_min (cadência de L1)]))</f>
         <v>1.536</v>
       </c>
-      <c r="G12" s="34"/>
-      <c r="I12" s="55" t="s">
+      <c r="G12" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B12,Table4[ref_id],Table4[família])</f>
+        <v>S</v>
+      </c>
+      <c r="H12" s="34" cm="1">
+        <f t="array" ref="H12">_xlfn.XLOOKUP(B12,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>1</v>
+      </c>
+      <c r="J12" s="55" t="s">
         <v>129</v>
       </c>
-      <c r="J12" s="55" t="s">
+      <c r="K12" s="55" t="s">
         <v>305</v>
       </c>
-      <c r="K12" s="55" t="s">
+      <c r="L12" s="55" t="s">
         <v>510</v>
       </c>
-      <c r="L12" s="55" t="s">
+      <c r="M12" s="55" t="s">
         <v>528</v>
       </c>
-    </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N12" s="75"/>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B13" s="34" t="s">
         <v>372</v>
       </c>
@@ -19069,7 +19189,7 @@
         <v>288</v>
       </c>
       <c r="D13" s="37">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="E13" s="60">
         <v>2</v>
@@ -19078,21 +19198,29 @@
         <f>C13*E13/76</f>
         <v>7.5789473684210522</v>
       </c>
-      <c r="G13" s="34"/>
-      <c r="I13" s="55" t="s">
+      <c r="G13" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B13,Table4[ref_id],Table4[família])</f>
+        <v>BW</v>
+      </c>
+      <c r="H13" s="34" cm="1">
+        <f t="array" ref="H13">_xlfn.XLOOKUP(B13,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>1</v>
+      </c>
+      <c r="J13" s="55" t="s">
         <v>152</v>
       </c>
-      <c r="J13" s="55" t="s">
+      <c r="K13" s="55" t="s">
         <v>328</v>
       </c>
-      <c r="K13" s="55" t="s">
+      <c r="L13" s="55" t="s">
         <v>406</v>
       </c>
-      <c r="L13" s="55" t="s">
+      <c r="M13" s="55" t="s">
         <v>527</v>
       </c>
-    </row>
-    <row r="14" spans="2:12" ht="12.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N13" s="75"/>
+    </row>
+    <row r="14" spans="2:14" ht="12.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="34" t="s">
         <v>293</v>
       </c>
@@ -19109,21 +19237,29 @@
         <f>C14*E14/(_xlfn.XLOOKUP(B14,Table4[ref_id],Table4[tempo_L1_prod_min (cadência de L1)]))</f>
         <v>0.84</v>
       </c>
-      <c r="G14" s="34"/>
-      <c r="I14" s="55" t="s">
+      <c r="G14" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B14,Table4[ref_id],Table4[família])</f>
+        <v>BG</v>
+      </c>
+      <c r="H14" s="34" cm="1">
+        <f t="array" ref="H14">_xlfn.XLOOKUP(B14,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>1</v>
+      </c>
+      <c r="J14" s="55" t="s">
         <v>188</v>
       </c>
-      <c r="J14" s="55" t="s">
+      <c r="K14" s="55" t="s">
         <v>364</v>
       </c>
-      <c r="K14" s="55" t="s">
+      <c r="L14" s="55" t="s">
         <v>406</v>
       </c>
-      <c r="L14" s="55" t="s">
+      <c r="M14" s="55" t="s">
         <v>528</v>
       </c>
-    </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N14" s="75"/>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B15" s="34" t="s">
         <v>333</v>
       </c>
@@ -19131,7 +19267,7 @@
         <v>63</v>
       </c>
       <c r="D15" s="37">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="E15" s="60">
         <v>4</v>
@@ -19140,21 +19276,29 @@
         <f>C15*E15/(_xlfn.XLOOKUP(B15,Table4[ref_id],Table4[tempo_L1_prod_min (cadência de L1)]))</f>
         <v>0.84</v>
       </c>
-      <c r="G15" s="34"/>
-      <c r="I15" s="55" t="s">
+      <c r="G15" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B15,Table4[ref_id],Table4[família])</f>
+        <v>CH</v>
+      </c>
+      <c r="H15" s="34" cm="1">
+        <f t="array" ref="H15">_xlfn.XLOOKUP(B15,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="55" t="s">
         <v>196</v>
       </c>
-      <c r="J15" s="55" t="s">
+      <c r="K15" s="55" t="s">
         <v>372</v>
       </c>
-      <c r="K15" s="55" t="s">
+      <c r="L15" s="55" t="s">
         <v>406</v>
       </c>
-      <c r="L15" s="55" t="s">
+      <c r="M15" s="55" t="s">
         <v>528</v>
       </c>
-    </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N15" s="75"/>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B16" s="34" t="s">
         <v>514</v>
       </c>
@@ -19162,7 +19306,7 @@
         <v>938</v>
       </c>
       <c r="D16" s="37">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="E16" s="60">
         <v>4</v>
@@ -19171,21 +19315,29 @@
         <f>C16*E16/(_xlfn.XLOOKUP(B16,Table4[ref_id],Table4[tempo_L1_prod_min (cadência de L1)]))</f>
         <v>10.72</v>
       </c>
-      <c r="G16" s="34"/>
-      <c r="I16" s="55" t="s">
+      <c r="G16" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B16,Table4[ref_id],Table4[família])</f>
+        <v>B</v>
+      </c>
+      <c r="H16" s="34" cm="1">
+        <f t="array" ref="H16">_xlfn.XLOOKUP(B16,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>1</v>
+      </c>
+      <c r="J16" s="55" t="s">
         <v>116</v>
       </c>
-      <c r="J16" s="55" t="s">
+      <c r="K16" s="55" t="s">
         <v>293</v>
       </c>
-      <c r="K16" s="55" t="s">
+      <c r="L16" s="55" t="s">
         <v>406</v>
       </c>
-      <c r="L16" s="55" t="s">
+      <c r="M16" s="55" t="s">
         <v>527</v>
       </c>
-    </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N16" s="75"/>
+    </row>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B17" s="34" t="s">
         <v>321</v>
       </c>
@@ -19193,7 +19345,7 @@
         <v>360</v>
       </c>
       <c r="D17" s="37">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="E17" s="60">
         <v>3</v>
@@ -19202,21 +19354,29 @@
         <f>C17*E17/220</f>
         <v>4.9090909090909092</v>
       </c>
-      <c r="G17" s="34"/>
-      <c r="I17" s="55" t="s">
+      <c r="G17" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B17,Table4[ref_id],Table4[família])</f>
+        <v>X</v>
+      </c>
+      <c r="H17" s="34" cm="1">
+        <f t="array" ref="H17">_xlfn.XLOOKUP(B17,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>1</v>
+      </c>
+      <c r="J17" s="55" t="s">
         <v>157</v>
       </c>
-      <c r="J17" s="55" t="s">
+      <c r="K17" s="55" t="s">
         <v>333</v>
       </c>
-      <c r="K17" s="55" t="s">
+      <c r="L17" s="55" t="s">
         <v>526</v>
       </c>
-      <c r="L17" s="55" t="s">
+      <c r="M17" s="55" t="s">
         <v>527</v>
       </c>
-    </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N17" s="75"/>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B18" s="34" t="s">
         <v>261</v>
       </c>
@@ -19224,7 +19384,7 @@
         <v>64</v>
       </c>
       <c r="D18" s="37">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="E18" s="34">
         <v>4</v>
@@ -19233,22 +19393,30 @@
         <f>C18*E18/(_xlfn.XLOOKUP(B18,Table4[ref_id],Table4[tempo_L1_prod_min (cadência de L1)]))</f>
         <v>1.0666666666666667</v>
       </c>
-      <c r="G18" s="34"/>
-      <c r="H18" s="38"/>
-      <c r="I18" s="55" t="s">
+      <c r="G18" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B18,Table4[ref_id],Table4[família])</f>
+        <v>B</v>
+      </c>
+      <c r="H18" s="34" cm="1">
+        <f t="array" ref="H18">_xlfn.XLOOKUP(B18,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>1</v>
+      </c>
+      <c r="I18" s="38"/>
+      <c r="J18" s="55" t="s">
         <v>516</v>
       </c>
-      <c r="J18" s="55" t="s">
+      <c r="K18" s="55" t="s">
         <v>514</v>
       </c>
-      <c r="K18" s="55" t="s">
+      <c r="L18" s="55" t="s">
         <v>406</v>
       </c>
-      <c r="L18" s="55" t="s">
+      <c r="M18" s="55" t="s">
         <v>527</v>
       </c>
-    </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N18" s="75"/>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B19" s="34" t="s">
         <v>364</v>
       </c>
@@ -19256,7 +19424,7 @@
         <v>72</v>
       </c>
       <c r="D19" s="37">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="E19" s="34">
         <v>3</v>
@@ -19265,686 +19433,771 @@
         <f>C19*E19/220</f>
         <v>0.98181818181818181</v>
       </c>
-      <c r="G19" s="34"/>
-      <c r="H19" s="38"/>
-      <c r="I19" s="55" t="s">
+      <c r="G19" s="34" t="str">
+        <f>_xlfn.XLOOKUP(B19,Table4[ref_id],Table4[família])</f>
+        <v>PL</v>
+      </c>
+      <c r="H19" s="34" cm="1">
+        <f t="array" ref="H19">_xlfn.XLOOKUP(B19,Table4[ref_id],'2_REFERENCIAS'!$D$5:$D$192)</f>
+        <v>1</v>
+      </c>
+      <c r="I19" s="38"/>
+      <c r="J19" s="55" t="s">
         <v>532</v>
       </c>
-      <c r="J19" s="55" t="s">
+      <c r="K19" s="55" t="s">
         <v>321</v>
       </c>
-      <c r="K19" s="55" t="s">
+      <c r="L19" s="55" t="s">
         <v>406</v>
       </c>
-      <c r="L19" s="55" t="s">
+      <c r="M19" s="55" t="s">
         <v>528</v>
       </c>
-    </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="N19" s="75"/>
+    </row>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B20" s="34"/>
       <c r="C20" s="34"/>
       <c r="D20" s="34"/>
       <c r="E20" s="34"/>
       <c r="F20" s="34"/>
       <c r="G20" s="34"/>
-      <c r="H20" s="38"/>
-    </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H20" s="34"/>
+      <c r="I20" s="38"/>
+      <c r="M20" s="75"/>
+      <c r="N20" s="75"/>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B21" s="34"/>
       <c r="C21" s="34"/>
       <c r="D21" s="34"/>
       <c r="E21" s="34"/>
       <c r="F21" s="34"/>
       <c r="G21" s="34"/>
-      <c r="H21" s="38"/>
-    </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H21" s="34"/>
+      <c r="I21" s="38"/>
+      <c r="M21" s="75"/>
+      <c r="N21" s="75"/>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B22" s="34"/>
       <c r="C22" s="34"/>
       <c r="D22" s="34"/>
       <c r="E22" s="34"/>
       <c r="F22" s="34"/>
       <c r="G22" s="34"/>
-      <c r="H22" s="38"/>
-    </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H22" s="34"/>
+      <c r="I22" s="38"/>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B23" s="34"/>
       <c r="C23" s="34"/>
       <c r="D23" s="34"/>
       <c r="E23" s="34"/>
       <c r="F23" s="34"/>
       <c r="G23" s="34"/>
-      <c r="H23" s="38"/>
-    </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H23" s="34"/>
+      <c r="I23" s="38"/>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B24" s="34"/>
       <c r="C24" s="34"/>
       <c r="D24" s="34"/>
       <c r="E24" s="37"/>
       <c r="F24" s="57"/>
       <c r="G24" s="57"/>
-      <c r="H24" s="38"/>
-    </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H24" s="57"/>
+      <c r="I24" s="38"/>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B25" s="34"/>
       <c r="C25" s="34"/>
       <c r="D25" s="34"/>
       <c r="E25" s="37"/>
       <c r="F25" s="57"/>
       <c r="G25" s="57"/>
-      <c r="H25" s="38"/>
-    </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H25" s="57"/>
+      <c r="I25" s="38"/>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B26" s="34"/>
       <c r="C26" s="34"/>
       <c r="D26" s="34"/>
       <c r="E26" s="37"/>
       <c r="F26" s="57"/>
       <c r="G26" s="57"/>
-      <c r="H26" s="38"/>
-    </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H26" s="57"/>
+      <c r="I26" s="38"/>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B27" s="34"/>
       <c r="C27" s="34"/>
       <c r="D27" s="34"/>
       <c r="E27" s="37"/>
       <c r="F27" s="57"/>
       <c r="G27" s="57"/>
-      <c r="H27" s="38"/>
-    </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H27" s="57"/>
+      <c r="I27" s="38"/>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B28" s="34"/>
       <c r="C28" s="34"/>
       <c r="D28" s="34"/>
       <c r="E28" s="37"/>
       <c r="F28" s="57"/>
       <c r="G28" s="57"/>
-      <c r="H28" s="38"/>
-    </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H28" s="57"/>
+      <c r="I28" s="38"/>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B29" s="34"/>
       <c r="C29" s="34"/>
       <c r="D29" s="34"/>
       <c r="E29" s="37"/>
       <c r="F29" s="57"/>
       <c r="G29" s="57"/>
-      <c r="H29" s="38"/>
-    </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H29" s="57"/>
+      <c r="I29" s="38"/>
+    </row>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B30" s="34"/>
       <c r="C30" s="34"/>
       <c r="D30" s="34"/>
       <c r="E30" s="37"/>
       <c r="F30" s="57"/>
       <c r="G30" s="57"/>
-      <c r="H30" s="38"/>
-    </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H30" s="57"/>
+      <c r="I30" s="38"/>
+    </row>
+    <row r="31" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B31" s="34"/>
       <c r="C31" s="34"/>
       <c r="D31" s="34"/>
       <c r="E31" s="37"/>
       <c r="F31" s="57"/>
       <c r="G31" s="57"/>
-      <c r="H31" s="38"/>
-    </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H31" s="57"/>
+      <c r="I31" s="38"/>
+    </row>
+    <row r="32" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B32" s="34"/>
       <c r="C32" s="34"/>
       <c r="D32" s="34"/>
       <c r="E32" s="37"/>
       <c r="F32" s="57"/>
       <c r="G32" s="57"/>
-      <c r="H32" s="38"/>
-    </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H32" s="57"/>
+      <c r="I32" s="38"/>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B33" s="34"/>
       <c r="C33" s="34"/>
       <c r="D33" s="34"/>
       <c r="E33" s="37"/>
       <c r="F33" s="57"/>
       <c r="G33" s="57"/>
-      <c r="H33" s="38"/>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H33" s="57"/>
+      <c r="I33" s="38"/>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B34" s="34"/>
       <c r="C34" s="34"/>
       <c r="D34" s="34"/>
       <c r="E34" s="37"/>
       <c r="F34" s="57"/>
       <c r="G34" s="57"/>
-      <c r="H34" s="38"/>
-    </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H34" s="57"/>
+      <c r="I34" s="38"/>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B35" s="34"/>
       <c r="C35" s="34"/>
       <c r="D35" s="34"/>
       <c r="E35" s="37"/>
       <c r="F35" s="57"/>
       <c r="G35" s="57"/>
-      <c r="H35" s="38"/>
-    </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H35" s="57"/>
+      <c r="I35" s="38"/>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B36" s="34"/>
       <c r="C36" s="34"/>
       <c r="D36" s="34"/>
       <c r="E36" s="37"/>
       <c r="F36" s="57"/>
       <c r="G36" s="57"/>
-      <c r="H36" s="38"/>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H36" s="57"/>
+      <c r="I36" s="38"/>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B37" s="34"/>
       <c r="C37" s="34"/>
       <c r="D37" s="34"/>
       <c r="E37" s="37"/>
       <c r="F37" s="57"/>
       <c r="G37" s="57"/>
-      <c r="H37" s="38"/>
-    </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H37" s="57"/>
+      <c r="I37" s="38"/>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B38" s="34"/>
       <c r="C38" s="34"/>
       <c r="D38" s="34"/>
       <c r="E38" s="37"/>
       <c r="F38" s="57"/>
       <c r="G38" s="57"/>
-      <c r="H38" s="38"/>
-    </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H38" s="57"/>
+      <c r="I38" s="38"/>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B39" s="34"/>
       <c r="C39" s="34"/>
       <c r="D39" s="34"/>
       <c r="E39" s="37"/>
       <c r="F39" s="57"/>
       <c r="G39" s="57"/>
-      <c r="H39" s="38"/>
-    </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H39" s="57"/>
+      <c r="I39" s="38"/>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B40" s="34"/>
       <c r="C40" s="34"/>
       <c r="D40" s="34"/>
       <c r="E40" s="37"/>
       <c r="F40" s="57"/>
       <c r="G40" s="57"/>
-      <c r="H40" s="38"/>
-    </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H40" s="57"/>
+      <c r="I40" s="38"/>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B41" s="34"/>
       <c r="C41" s="34"/>
       <c r="D41" s="34"/>
       <c r="E41" s="37"/>
       <c r="F41" s="57"/>
       <c r="G41" s="57"/>
-      <c r="H41" s="38"/>
-    </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H41" s="57"/>
+      <c r="I41" s="38"/>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B42" s="34"/>
       <c r="C42" s="34"/>
       <c r="D42" s="34"/>
       <c r="E42" s="37"/>
       <c r="F42" s="57"/>
       <c r="G42" s="57"/>
-      <c r="H42" s="38"/>
-    </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H42" s="57"/>
+      <c r="I42" s="38"/>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B43" s="34"/>
       <c r="C43" s="34"/>
       <c r="D43" s="34"/>
       <c r="E43" s="37"/>
       <c r="F43" s="57"/>
       <c r="G43" s="57"/>
-      <c r="H43" s="38"/>
-    </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H43" s="57"/>
+      <c r="I43" s="38"/>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B44" s="34"/>
       <c r="C44" s="34"/>
       <c r="D44" s="34"/>
       <c r="E44" s="37"/>
       <c r="F44" s="57"/>
       <c r="G44" s="57"/>
-      <c r="H44" s="38"/>
-    </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H44" s="57"/>
+      <c r="I44" s="38"/>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B45" s="34"/>
       <c r="C45" s="34"/>
       <c r="D45" s="34"/>
       <c r="E45" s="37"/>
       <c r="F45" s="57"/>
       <c r="G45" s="57"/>
-      <c r="H45" s="38"/>
-    </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H45" s="57"/>
+      <c r="I45" s="38"/>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B46" s="34"/>
       <c r="C46" s="34"/>
       <c r="D46" s="34"/>
       <c r="E46" s="37"/>
       <c r="F46" s="57"/>
       <c r="G46" s="57"/>
-      <c r="H46" s="38"/>
-    </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H46" s="57"/>
+      <c r="I46" s="38"/>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B47" s="34"/>
       <c r="C47" s="34"/>
       <c r="D47" s="34"/>
       <c r="E47" s="37"/>
       <c r="F47" s="57"/>
       <c r="G47" s="57"/>
-      <c r="H47" s="38"/>
-    </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H47" s="57"/>
+      <c r="I47" s="38"/>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B48" s="34"/>
       <c r="C48" s="34"/>
       <c r="D48" s="34"/>
       <c r="E48" s="37"/>
       <c r="F48" s="57"/>
       <c r="G48" s="57"/>
-      <c r="H48" s="38"/>
-    </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H48" s="57"/>
+      <c r="I48" s="38"/>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B49" s="34"/>
       <c r="C49" s="34"/>
       <c r="D49" s="34"/>
       <c r="E49" s="37"/>
       <c r="F49" s="57"/>
       <c r="G49" s="57"/>
-      <c r="H49" s="38"/>
-    </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H49" s="57"/>
+      <c r="I49" s="38"/>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B50" s="34"/>
       <c r="C50" s="34"/>
       <c r="D50" s="34"/>
       <c r="E50" s="37"/>
       <c r="F50" s="57"/>
       <c r="G50" s="57"/>
-      <c r="H50" s="38"/>
-    </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H50" s="57"/>
+      <c r="I50" s="38"/>
+    </row>
+    <row r="51" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B51" s="34"/>
       <c r="C51" s="34"/>
       <c r="D51" s="34"/>
       <c r="E51" s="37"/>
       <c r="F51" s="57"/>
       <c r="G51" s="57"/>
-      <c r="H51" s="38"/>
-    </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H51" s="57"/>
+      <c r="I51" s="38"/>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B52" s="34"/>
       <c r="C52" s="34"/>
       <c r="D52" s="34"/>
       <c r="E52" s="37"/>
       <c r="F52" s="57"/>
       <c r="G52" s="57"/>
-      <c r="H52" s="38"/>
-    </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H52" s="57"/>
+      <c r="I52" s="38"/>
+    </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B53" s="34"/>
       <c r="C53" s="34"/>
       <c r="D53" s="34"/>
       <c r="E53" s="37"/>
       <c r="F53" s="57"/>
       <c r="G53" s="57"/>
-      <c r="H53" s="38"/>
-    </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H53" s="57"/>
+      <c r="I53" s="38"/>
+    </row>
+    <row r="54" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B54" s="34"/>
       <c r="C54" s="34"/>
       <c r="D54" s="34"/>
       <c r="E54" s="37"/>
       <c r="F54" s="57"/>
       <c r="G54" s="57"/>
-      <c r="H54" s="38"/>
-    </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H54" s="57"/>
+      <c r="I54" s="38"/>
+    </row>
+    <row r="55" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B55" s="34"/>
       <c r="C55" s="34"/>
       <c r="D55" s="34"/>
       <c r="E55" s="37"/>
       <c r="F55" s="57"/>
       <c r="G55" s="57"/>
-      <c r="H55" s="38"/>
-    </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H55" s="57"/>
+      <c r="I55" s="38"/>
+    </row>
+    <row r="56" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B56" s="34"/>
       <c r="C56" s="34"/>
       <c r="D56" s="34"/>
       <c r="E56" s="37"/>
       <c r="F56" s="57"/>
       <c r="G56" s="57"/>
-      <c r="H56" s="38"/>
-    </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H56" s="57"/>
+      <c r="I56" s="38"/>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B57" s="34"/>
       <c r="C57" s="34"/>
       <c r="D57" s="34"/>
       <c r="E57" s="37"/>
       <c r="F57" s="57"/>
       <c r="G57" s="57"/>
-      <c r="H57" s="38"/>
-    </row>
-    <row r="58" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H57" s="57"/>
+      <c r="I57" s="38"/>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B58" s="34"/>
       <c r="C58" s="34"/>
       <c r="D58" s="34"/>
       <c r="E58" s="37"/>
       <c r="F58" s="57"/>
       <c r="G58" s="57"/>
-      <c r="H58" s="38"/>
-    </row>
-    <row r="59" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H58" s="57"/>
+      <c r="I58" s="38"/>
+    </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B59" s="34"/>
       <c r="C59" s="34"/>
       <c r="D59" s="34"/>
       <c r="E59" s="37"/>
       <c r="F59" s="57"/>
       <c r="G59" s="57"/>
-      <c r="H59" s="38"/>
-    </row>
-    <row r="60" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H59" s="57"/>
+      <c r="I59" s="38"/>
+    </row>
+    <row r="60" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B60" s="34"/>
       <c r="C60" s="34"/>
       <c r="D60" s="34"/>
       <c r="E60" s="37"/>
       <c r="F60" s="57"/>
       <c r="G60" s="57"/>
-      <c r="H60" s="38"/>
-    </row>
-    <row r="61" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H60" s="57"/>
+      <c r="I60" s="38"/>
+    </row>
+    <row r="61" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B61" s="34"/>
       <c r="C61" s="34"/>
       <c r="D61" s="34"/>
       <c r="E61" s="37"/>
       <c r="F61" s="57"/>
       <c r="G61" s="57"/>
-      <c r="H61" s="38"/>
-    </row>
-    <row r="62" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H61" s="57"/>
+      <c r="I61" s="38"/>
+    </row>
+    <row r="62" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B62" s="34"/>
       <c r="C62" s="34"/>
       <c r="D62" s="34"/>
       <c r="E62" s="37"/>
       <c r="F62" s="57"/>
       <c r="G62" s="57"/>
-      <c r="H62" s="38"/>
-    </row>
-    <row r="63" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H62" s="57"/>
+      <c r="I62" s="38"/>
+    </row>
+    <row r="63" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B63" s="34"/>
       <c r="C63" s="34"/>
       <c r="D63" s="34"/>
       <c r="E63" s="37"/>
       <c r="F63" s="57"/>
       <c r="G63" s="57"/>
-      <c r="H63" s="38"/>
-    </row>
-    <row r="64" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="H63" s="57"/>
+      <c r="I63" s="38"/>
+    </row>
+    <row r="64" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B64" s="34"/>
       <c r="C64" s="34"/>
       <c r="D64" s="34"/>
       <c r="E64" s="37"/>
       <c r="F64" s="57"/>
       <c r="G64" s="57"/>
-      <c r="H64" s="38"/>
-    </row>
-    <row r="65" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H64" s="57"/>
+      <c r="I64" s="38"/>
+    </row>
+    <row r="65" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B65" s="34"/>
       <c r="C65" s="34"/>
       <c r="D65" s="34"/>
       <c r="E65" s="37"/>
       <c r="F65" s="57"/>
       <c r="G65" s="57"/>
-      <c r="H65" s="38"/>
-    </row>
-    <row r="66" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H65" s="57"/>
+      <c r="I65" s="38"/>
+    </row>
+    <row r="66" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B66" s="34"/>
       <c r="C66" s="34"/>
       <c r="D66" s="34"/>
       <c r="E66" s="37"/>
       <c r="F66" s="57"/>
       <c r="G66" s="57"/>
-      <c r="H66" s="38"/>
-    </row>
-    <row r="67" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H66" s="57"/>
+      <c r="I66" s="38"/>
+    </row>
+    <row r="67" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B67" s="34"/>
       <c r="C67" s="34"/>
       <c r="D67" s="34"/>
       <c r="E67" s="37"/>
       <c r="F67" s="57"/>
       <c r="G67" s="57"/>
-      <c r="H67" s="38"/>
-    </row>
-    <row r="68" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H67" s="57"/>
+      <c r="I67" s="38"/>
+    </row>
+    <row r="68" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B68" s="34"/>
       <c r="C68" s="34"/>
       <c r="D68" s="34"/>
       <c r="E68" s="37"/>
       <c r="F68" s="57"/>
       <c r="G68" s="57"/>
-      <c r="H68" s="38"/>
-      <c r="L68" t="s">
+      <c r="H68" s="57"/>
+      <c r="I68" s="38"/>
+      <c r="M68" t="s">
         <v>527</v>
       </c>
     </row>
-    <row r="69" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B69" s="34"/>
       <c r="C69" s="34"/>
       <c r="D69" s="34"/>
       <c r="E69" s="37"/>
       <c r="F69" s="57"/>
       <c r="G69" s="57"/>
-      <c r="H69" s="38"/>
-    </row>
-    <row r="70" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H69" s="57"/>
+      <c r="I69" s="38"/>
+    </row>
+    <row r="70" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B70" s="34"/>
       <c r="C70" s="34"/>
       <c r="D70" s="34"/>
       <c r="E70" s="37"/>
       <c r="F70" s="57"/>
       <c r="G70" s="57"/>
-      <c r="H70" s="38"/>
-    </row>
-    <row r="71" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H70" s="57"/>
+      <c r="I70" s="38"/>
+    </row>
+    <row r="71" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B71" s="34"/>
       <c r="C71" s="34"/>
       <c r="D71" s="34"/>
       <c r="E71" s="37"/>
       <c r="F71" s="57"/>
       <c r="G71" s="57"/>
-      <c r="H71" s="38"/>
-    </row>
-    <row r="72" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H71" s="57"/>
+      <c r="I71" s="38"/>
+    </row>
+    <row r="72" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B72" s="34"/>
       <c r="C72" s="34"/>
       <c r="D72" s="34"/>
       <c r="E72" s="37"/>
       <c r="F72" s="57"/>
       <c r="G72" s="57"/>
-      <c r="H72" s="38"/>
-    </row>
-    <row r="73" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H72" s="57"/>
+      <c r="I72" s="38"/>
+    </row>
+    <row r="73" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B73" s="34"/>
       <c r="C73" s="34"/>
       <c r="D73" s="34"/>
       <c r="E73" s="37"/>
       <c r="F73" s="57"/>
       <c r="G73" s="57"/>
-      <c r="H73" s="38"/>
-    </row>
-    <row r="74" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H73" s="57"/>
+      <c r="I73" s="38"/>
+    </row>
+    <row r="74" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B74" s="34"/>
       <c r="C74" s="34"/>
       <c r="D74" s="34"/>
       <c r="E74" s="37"/>
       <c r="F74" s="57"/>
       <c r="G74" s="57"/>
-      <c r="H74" s="38"/>
-    </row>
-    <row r="75" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H74" s="57"/>
+      <c r="I74" s="38"/>
+    </row>
+    <row r="75" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B75" s="34"/>
       <c r="C75" s="34"/>
       <c r="D75" s="34"/>
       <c r="E75" s="37"/>
       <c r="F75" s="57"/>
       <c r="G75" s="57"/>
-      <c r="H75" s="38"/>
-    </row>
-    <row r="76" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H75" s="57"/>
+      <c r="I75" s="38"/>
+    </row>
+    <row r="76" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B76" s="34"/>
       <c r="C76" s="34"/>
       <c r="D76" s="34"/>
       <c r="E76" s="37"/>
       <c r="F76" s="57"/>
       <c r="G76" s="57"/>
-      <c r="H76" s="38"/>
-    </row>
-    <row r="77" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H76" s="57"/>
+      <c r="I76" s="38"/>
+    </row>
+    <row r="77" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B77" s="34"/>
       <c r="C77" s="34"/>
       <c r="D77" s="34"/>
       <c r="E77" s="37"/>
       <c r="F77" s="57"/>
       <c r="G77" s="57"/>
-      <c r="H77" s="38"/>
-    </row>
-    <row r="78" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H77" s="57"/>
+      <c r="I77" s="38"/>
+    </row>
+    <row r="78" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B78" s="34"/>
       <c r="C78" s="34"/>
       <c r="D78" s="34"/>
       <c r="E78" s="37"/>
       <c r="F78" s="57"/>
       <c r="G78" s="57"/>
-      <c r="H78" s="38"/>
-    </row>
-    <row r="79" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H78" s="57"/>
+      <c r="I78" s="38"/>
+    </row>
+    <row r="79" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B79" s="34"/>
       <c r="C79" s="34"/>
       <c r="D79" s="34"/>
       <c r="E79" s="37"/>
       <c r="F79" s="57"/>
       <c r="G79" s="57"/>
-      <c r="H79" s="38"/>
-    </row>
-    <row r="80" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H79" s="57"/>
+      <c r="I79" s="38"/>
+    </row>
+    <row r="80" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B80" s="34"/>
       <c r="C80" s="34"/>
       <c r="D80" s="34"/>
       <c r="E80" s="37"/>
       <c r="F80" s="57"/>
       <c r="G80" s="57"/>
-      <c r="H80" s="38"/>
-      <c r="L80" t="s">
+      <c r="H80" s="57"/>
+      <c r="I80" s="38"/>
+      <c r="M80" t="s">
         <v>527</v>
       </c>
     </row>
-    <row r="81" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B81" s="34"/>
       <c r="C81" s="34"/>
       <c r="D81" s="34"/>
       <c r="E81" s="37"/>
       <c r="F81" s="57"/>
       <c r="G81" s="57"/>
-      <c r="H81" s="38"/>
-    </row>
-    <row r="82" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H81" s="57"/>
+      <c r="I81" s="38"/>
+    </row>
+    <row r="82" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B82" s="34"/>
       <c r="C82" s="34"/>
       <c r="D82" s="34"/>
       <c r="E82" s="37"/>
       <c r="F82" s="57"/>
       <c r="G82" s="57"/>
-      <c r="H82" s="38"/>
-    </row>
-    <row r="83" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H82" s="57"/>
+      <c r="I82" s="38"/>
+    </row>
+    <row r="83" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B83" s="34"/>
       <c r="C83" s="34"/>
       <c r="D83" s="34"/>
       <c r="E83" s="37"/>
       <c r="F83" s="57"/>
       <c r="G83" s="57"/>
-      <c r="H83" s="38"/>
-    </row>
-    <row r="84" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H83" s="57"/>
+      <c r="I83" s="38"/>
+    </row>
+    <row r="84" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B84" s="34"/>
       <c r="C84" s="34"/>
       <c r="D84" s="34"/>
       <c r="E84" s="37"/>
       <c r="F84" s="57"/>
       <c r="G84" s="57"/>
-      <c r="H84" s="38"/>
-    </row>
-    <row r="85" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H84" s="57"/>
+      <c r="I84" s="38"/>
+    </row>
+    <row r="85" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B85" s="34"/>
       <c r="C85" s="34"/>
       <c r="D85" s="34"/>
       <c r="E85" s="37"/>
       <c r="F85" s="57"/>
       <c r="G85" s="57"/>
-      <c r="H85" s="38"/>
-    </row>
-    <row r="86" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H85" s="57"/>
+      <c r="I85" s="38"/>
+    </row>
+    <row r="86" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B86" s="34"/>
       <c r="C86" s="34"/>
       <c r="D86" s="34"/>
       <c r="E86" s="37"/>
       <c r="F86" s="57"/>
       <c r="G86" s="57"/>
-      <c r="H86" s="38"/>
-    </row>
-    <row r="87" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H86" s="57"/>
+      <c r="I86" s="38"/>
+    </row>
+    <row r="87" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B87" s="34"/>
       <c r="C87" s="34"/>
       <c r="D87" s="34"/>
       <c r="E87" s="37"/>
       <c r="F87" s="57"/>
       <c r="G87" s="57"/>
-      <c r="H87" s="38"/>
-      <c r="L87" t="s">
+      <c r="H87" s="57"/>
+      <c r="I87" s="38"/>
+      <c r="M87" t="s">
         <v>528</v>
       </c>
     </row>
-    <row r="88" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B88" s="34"/>
       <c r="C88" s="34"/>
       <c r="D88" s="34"/>
       <c r="E88" s="37"/>
       <c r="F88" s="57"/>
       <c r="G88" s="57"/>
-      <c r="H88" s="38"/>
-    </row>
-    <row r="89" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H88" s="57"/>
+      <c r="I88" s="38"/>
+    </row>
+    <row r="89" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B89" s="34"/>
       <c r="C89" s="34"/>
       <c r="D89" s="34"/>
       <c r="E89" s="37"/>
       <c r="F89" s="57"/>
       <c r="G89" s="57"/>
-      <c r="H89" s="38"/>
-    </row>
-    <row r="90" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H89" s="57"/>
+      <c r="I89" s="38"/>
+    </row>
+    <row r="90" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B90" s="34"/>
       <c r="C90" s="34"/>
       <c r="D90" s="34"/>
       <c r="E90" s="37"/>
       <c r="F90" s="57"/>
       <c r="G90" s="57"/>
-    </row>
-    <row r="91" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H90" s="57"/>
+    </row>
+    <row r="91" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B91" s="34"/>
       <c r="C91" s="34"/>
       <c r="D91" s="34"/>
       <c r="E91" s="37"/>
       <c r="F91" s="57"/>
       <c r="G91" s="57"/>
-    </row>
-    <row r="92" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="H91" s="57"/>
+    </row>
+    <row r="92" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B92" s="34"/>
       <c r="C92" s="34"/>
       <c r="D92" s="34"/>
       <c r="E92" s="37"/>
       <c r="F92" s="57"/>
       <c r="G92" s="57"/>
-    </row>
-    <row r="111" spans="12:12" x14ac:dyDescent="0.35">
-      <c r="L111" t="s">
+      <c r="H92" s="57"/>
+    </row>
+    <row r="111" spans="13:13" x14ac:dyDescent="0.35">
+      <c r="M111" t="s">
         <v>527</v>
       </c>
     </row>
@@ -19953,6 +20206,9 @@
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B1:E1"/>
   </mergeCells>
+  <conditionalFormatting sqref="B5:B19">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19995,7 +20251,9 @@
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" s="32"/>
+      <c r="A7" s="32">
+        <v>46183</v>
+      </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" s="32"/>

</xml_diff>

<commit_message>
Refactor genetic algorithm integration with Optuna for hyperparameter tuning; enhance evaluator functions for better scheduling and operator management; update dashboard for improved user input handling and reporting; remove legacy Optuna script and add results saving functionality.
</commit_message>
<xml_diff>
--- a/Inputs_Doceleia_small.xlsx
+++ b/Inputs_Doceleia_small.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kaizen\Documents\tese\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DD3C7F4-9F38-4D26-9DCD-73C5A47648A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CFE5089-05DC-4B71-819D-635EDB0A152E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2890,6 +2890,7 @@
     <xf numFmtId="1" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2899,16 +2900,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2926,7 +2927,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4029,11 +4029,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -4065,11 +4065,11 @@
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="64" t="s">
+      <c r="A6" s="69" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="65"/>
-      <c r="C6" s="65"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
     </row>
     <row r="7" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
@@ -4102,11 +4102,11 @@
       <c r="C9" s="3"/>
     </row>
     <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="64" t="s">
+      <c r="A11" s="69" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="65"/>
-      <c r="C11" s="65"/>
+      <c r="B11" s="66"/>
+      <c r="C11" s="66"/>
     </row>
     <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
@@ -4130,11 +4130,11 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="64" t="s">
+      <c r="A15" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="65"/>
-      <c r="C15" s="65"/>
+      <c r="B15" s="66"/>
+      <c r="C15" s="66"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
@@ -4216,11 +4216,11 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" s="64" t="s">
+      <c r="A24" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="B24" s="65"/>
-      <c r="C24" s="65"/>
+      <c r="B24" s="66"/>
+      <c r="C24" s="66"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
@@ -4300,11 +4300,11 @@
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A33" s="64" t="s">
+      <c r="A33" s="69" t="s">
         <v>21</v>
       </c>
-      <c r="B33" s="65"/>
-      <c r="C33" s="65"/>
+      <c r="B33" s="66"/>
+      <c r="C33" s="66"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="12" t="s">
@@ -4319,33 +4319,33 @@
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A37" s="72" t="s">
+      <c r="A37" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="B37" s="65"/>
-      <c r="C37" s="65"/>
+      <c r="B37" s="66"/>
+      <c r="C37" s="66"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A39" s="71" t="s">
+      <c r="A39" s="72" t="s">
         <v>42</v>
       </c>
       <c r="B39" s="68"/>
       <c r="C39" s="68"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A40" s="70" t="s">
+      <c r="A40" s="71" t="s">
         <v>24</v>
       </c>
       <c r="B40" s="68"/>
       <c r="C40" s="68"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A41" s="70"/>
+      <c r="A41" s="71"/>
       <c r="B41" s="68"/>
       <c r="C41" s="68"/>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A42" s="69" t="s">
+      <c r="A42" s="70" t="s">
         <v>25</v>
       </c>
       <c r="B42" s="68"/>
@@ -4359,29 +4359,34 @@
       <c r="C43" s="68"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A44" s="70" t="s">
+      <c r="A44" s="71" t="s">
         <v>26</v>
       </c>
       <c r="B44" s="68"/>
       <c r="C44" s="68"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A45" s="66"/>
-      <c r="B45" s="65"/>
-      <c r="C45" s="65"/>
+      <c r="A45" s="65"/>
+      <c r="B45" s="66"/>
+      <c r="C45" s="66"/>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A46" s="66"/>
-      <c r="B46" s="65"/>
-      <c r="C46" s="65"/>
+      <c r="A46" s="65"/>
+      <c r="B46" s="66"/>
+      <c r="C46" s="66"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A47" s="66"/>
-      <c r="B47" s="65"/>
-      <c r="C47" s="65"/>
+      <c r="A47" s="65"/>
+      <c r="B47" s="66"/>
+      <c r="C47" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A46:C46"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A43:C43"/>
@@ -4393,11 +4398,6 @@
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="A40:C40"/>
     <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A46:C46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4429,44 +4429,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
     </row>
     <row r="2" spans="1:17" ht="50" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="74" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="73"/>
-      <c r="M2" s="73"/>
-      <c r="N2" s="73"/>
-      <c r="O2" s="73"/>
-      <c r="P2" s="73"/>
-      <c r="Q2" s="73"/>
+      <c r="B2" s="74"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="74"/>
+      <c r="I2" s="74"/>
+      <c r="J2" s="74"/>
+      <c r="K2" s="74"/>
+      <c r="L2" s="74"/>
+      <c r="M2" s="74"/>
+      <c r="N2" s="74"/>
+      <c r="O2" s="74"/>
+      <c r="P2" s="74"/>
+      <c r="Q2" s="74"/>
     </row>
     <row r="4" spans="1:17" ht="31" x14ac:dyDescent="0.35">
       <c r="A4" s="15" t="s">
@@ -14698,109 +14698,109 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
+      <c r="P1" s="63"/>
+      <c r="Q1" s="63"/>
+      <c r="R1" s="63"/>
+      <c r="S1" s="63"/>
+      <c r="T1" s="63"/>
+      <c r="U1" s="63"/>
+      <c r="V1" s="63"/>
+      <c r="W1" s="63"/>
+      <c r="X1" s="63"/>
+      <c r="Y1" s="63"/>
+      <c r="Z1" s="63"/>
+      <c r="AA1" s="63"/>
+      <c r="AB1" s="63"/>
+      <c r="AC1" s="63"/>
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.35">
-      <c r="A2" s="61" t="s">
+      <c r="A2" s="62" t="s">
         <v>400</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
-      <c r="L2" s="62"/>
-      <c r="M2" s="62"/>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62"/>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62"/>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62"/>
-      <c r="V2" s="62"/>
-      <c r="W2" s="62"/>
-      <c r="X2" s="62"/>
-      <c r="Y2" s="62"/>
-      <c r="Z2" s="62"/>
-      <c r="AA2" s="62"/>
-      <c r="AB2" s="62"/>
-      <c r="AC2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
+      <c r="K2" s="63"/>
+      <c r="L2" s="63"/>
+      <c r="M2" s="63"/>
+      <c r="N2" s="63"/>
+      <c r="O2" s="63"/>
+      <c r="P2" s="63"/>
+      <c r="Q2" s="63"/>
+      <c r="R2" s="63"/>
+      <c r="S2" s="63"/>
+      <c r="T2" s="63"/>
+      <c r="U2" s="63"/>
+      <c r="V2" s="63"/>
+      <c r="W2" s="63"/>
+      <c r="X2" s="63"/>
+      <c r="Y2" s="63"/>
+      <c r="Z2" s="63"/>
+      <c r="AA2" s="63"/>
+      <c r="AB2" s="63"/>
+      <c r="AC2" s="63"/>
     </row>
     <row r="3" spans="1:38" ht="32" x14ac:dyDescent="0.7">
-      <c r="B3" s="74" t="s">
+      <c r="B3" s="75" t="s">
         <v>511</v>
       </c>
-      <c r="C3" s="74"/>
-      <c r="D3" s="74"/>
-      <c r="E3" s="74"/>
-      <c r="F3" s="74"/>
-      <c r="G3" s="74"/>
-      <c r="H3" s="74"/>
-      <c r="I3" s="74"/>
-      <c r="J3" s="74"/>
-      <c r="K3" s="74"/>
-      <c r="L3" s="74"/>
-      <c r="M3" s="74"/>
-      <c r="N3" s="74"/>
-      <c r="O3" s="74"/>
-      <c r="P3" s="74"/>
-      <c r="Q3" s="74"/>
-      <c r="R3" s="74"/>
-      <c r="S3" s="74"/>
-      <c r="T3" s="74"/>
-      <c r="U3" s="74"/>
-      <c r="V3" s="74"/>
-      <c r="W3" s="74"/>
-      <c r="X3" s="74"/>
-      <c r="Y3" s="74"/>
-      <c r="Z3" s="74"/>
-      <c r="AA3" s="74"/>
-      <c r="AB3" s="74"/>
-      <c r="AC3" s="74"/>
-      <c r="AD3" s="74"/>
-      <c r="AE3" s="74"/>
-      <c r="AF3" s="74"/>
-      <c r="AG3" s="74"/>
-      <c r="AH3" s="74"/>
-      <c r="AI3" s="74"/>
-      <c r="AJ3" s="74"/>
+      <c r="C3" s="75"/>
+      <c r="D3" s="75"/>
+      <c r="E3" s="75"/>
+      <c r="F3" s="75"/>
+      <c r="G3" s="75"/>
+      <c r="H3" s="75"/>
+      <c r="I3" s="75"/>
+      <c r="J3" s="75"/>
+      <c r="K3" s="75"/>
+      <c r="L3" s="75"/>
+      <c r="M3" s="75"/>
+      <c r="N3" s="75"/>
+      <c r="O3" s="75"/>
+      <c r="P3" s="75"/>
+      <c r="Q3" s="75"/>
+      <c r="R3" s="75"/>
+      <c r="S3" s="75"/>
+      <c r="T3" s="75"/>
+      <c r="U3" s="75"/>
+      <c r="V3" s="75"/>
+      <c r="W3" s="75"/>
+      <c r="X3" s="75"/>
+      <c r="Y3" s="75"/>
+      <c r="Z3" s="75"/>
+      <c r="AA3" s="75"/>
+      <c r="AB3" s="75"/>
+      <c r="AC3" s="75"/>
+      <c r="AD3" s="75"/>
+      <c r="AE3" s="75"/>
+      <c r="AF3" s="75"/>
+      <c r="AG3" s="75"/>
+      <c r="AH3" s="75"/>
+      <c r="AI3" s="75"/>
+      <c r="AJ3" s="75"/>
     </row>
     <row r="4" spans="1:38" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
@@ -18803,12 +18803,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="B1" s="63" t="s">
+      <c r="B1" s="64" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
@@ -18818,12 +18818,12 @@
       </c>
     </row>
     <row r="2" spans="2:14" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="62" t="s">
         <v>404</v>
       </c>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
       <c r="F2" s="59" t="s">
         <v>529</v>
       </c>
@@ -18841,8 +18841,8 @@
       </c>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="M3" s="75"/>
-      <c r="N3" s="75"/>
+      <c r="M3" s="61"/>
+      <c r="N3" s="61"/>
     </row>
     <row r="4" spans="2:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B4" s="35" t="s">
@@ -18866,8 +18866,8 @@
       <c r="H4" s="56" t="s">
         <v>535</v>
       </c>
-      <c r="M4" s="75"/>
-      <c r="N4" s="75"/>
+      <c r="M4" s="61"/>
+      <c r="N4" s="61"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B5" s="34" t="s">
@@ -18906,7 +18906,7 @@
       <c r="M5" s="55" t="s">
         <v>527</v>
       </c>
-      <c r="N5" s="75"/>
+      <c r="N5" s="61"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B6" s="34" t="s">
@@ -18945,7 +18945,7 @@
       <c r="M6" s="55" t="s">
         <v>528</v>
       </c>
-      <c r="N6" s="75"/>
+      <c r="N6" s="61"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B7" s="34" t="s">
@@ -18984,7 +18984,7 @@
       <c r="M7" s="55" t="s">
         <v>528</v>
       </c>
-      <c r="N7" s="75"/>
+      <c r="N7" s="61"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B8" s="34" t="s">
@@ -19023,7 +19023,7 @@
       <c r="M8" s="55" t="s">
         <v>527</v>
       </c>
-      <c r="N8" s="75"/>
+      <c r="N8" s="61"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B9" s="34" t="s">
@@ -19062,7 +19062,7 @@
       <c r="M9" s="55" t="s">
         <v>527</v>
       </c>
-      <c r="N9" s="75"/>
+      <c r="N9" s="61"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B10" s="34" t="s">
@@ -19101,7 +19101,7 @@
       <c r="M10" s="55" t="s">
         <v>527</v>
       </c>
-      <c r="N10" s="75"/>
+      <c r="N10" s="61"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B11" s="34" t="s">
@@ -19140,7 +19140,7 @@
       <c r="M11" s="55" t="s">
         <v>527</v>
       </c>
-      <c r="N11" s="75"/>
+      <c r="N11" s="61"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B12" s="34" t="s">
@@ -19179,7 +19179,7 @@
       <c r="M12" s="55" t="s">
         <v>528</v>
       </c>
-      <c r="N12" s="75"/>
+      <c r="N12" s="61"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B13" s="34" t="s">
@@ -19218,7 +19218,7 @@
       <c r="M13" s="55" t="s">
         <v>527</v>
       </c>
-      <c r="N13" s="75"/>
+      <c r="N13" s="61"/>
     </row>
     <row r="14" spans="2:14" ht="12.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="34" t="s">
@@ -19257,7 +19257,7 @@
       <c r="M14" s="55" t="s">
         <v>528</v>
       </c>
-      <c r="N14" s="75"/>
+      <c r="N14" s="61"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B15" s="34" t="s">
@@ -19296,7 +19296,7 @@
       <c r="M15" s="55" t="s">
         <v>528</v>
       </c>
-      <c r="N15" s="75"/>
+      <c r="N15" s="61"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B16" s="34" t="s">
@@ -19335,7 +19335,7 @@
       <c r="M16" s="55" t="s">
         <v>527</v>
       </c>
-      <c r="N16" s="75"/>
+      <c r="N16" s="61"/>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B17" s="34" t="s">
@@ -19374,7 +19374,7 @@
       <c r="M17" s="55" t="s">
         <v>527</v>
       </c>
-      <c r="N17" s="75"/>
+      <c r="N17" s="61"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B18" s="34" t="s">
@@ -19414,7 +19414,7 @@
       <c r="M18" s="55" t="s">
         <v>527</v>
       </c>
-      <c r="N18" s="75"/>
+      <c r="N18" s="61"/>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B19" s="34" t="s">
@@ -19454,7 +19454,7 @@
       <c r="M19" s="55" t="s">
         <v>528</v>
       </c>
-      <c r="N19" s="75"/>
+      <c r="N19" s="61"/>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B20" s="34"/>
@@ -19465,8 +19465,8 @@
       <c r="G20" s="34"/>
       <c r="H20" s="34"/>
       <c r="I20" s="38"/>
-      <c r="M20" s="75"/>
-      <c r="N20" s="75"/>
+      <c r="M20" s="61"/>
+      <c r="N20" s="61"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B21" s="34"/>
@@ -19477,8 +19477,8 @@
       <c r="G21" s="34"/>
       <c r="H21" s="34"/>
       <c r="I21" s="38"/>
-      <c r="M21" s="75"/>
-      <c r="N21" s="75"/>
+      <c r="M21" s="61"/>
+      <c r="N21" s="61"/>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B22" s="34"/>

</xml_diff>